<commit_message>
compoff non teaching working
</commit_message>
<xml_diff>
--- a/files/holiday_final.xlsx
+++ b/files/holiday_final.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="8">
   <si>
     <t>holidayName</t>
   </si>
@@ -33,16 +33,13 @@
     <t>description</t>
   </si>
   <si>
-    <t>Test</t>
-  </si>
-  <si>
     <t>applicableEmployeeCategories</t>
   </si>
   <si>
-    <t xml:space="preserve">test1 </t>
-  </si>
-  <si>
-    <t>Teaching</t>
+    <t>Teaching,Non-Teaching</t>
+  </si>
+  <si>
+    <t>Sample</t>
   </si>
 </sst>
 </file>
@@ -405,7 +402,7 @@
         <v>4</v>
       </c>
       <c r="E1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -419,10 +416,10 @@
         <v>3</v>
       </c>
       <c r="D2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>